<commit_message>
Actualizacion automatica Informe Semanal DEX
</commit_message>
<xml_diff>
--- a/excel/atipana-dex-s-a-c_ccc.xlsx
+++ b/excel/atipana-dex-s-a-c_ccc.xlsx
@@ -1769,16 +1769,16 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>74910</v>
+        <v>77541</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>C004174759</t>
+          <t>C004240376</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>C004174759 - BECERRA SOUZA JORGE ENRRIQUE</t>
+          <t>C004240376 - IGNACIO CARDENAS REGINALDA</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>S17848019</t>
+          <t>S17848813</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1842,11 +1842,11 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R12" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1868,7 +1868,7 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -1878,23 +1878,23 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más confianza en la entrega</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>77156</v>
+        <v>74910</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>C004221411</t>
+          <t>C004174759</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>C004221411 - BELLO OBREGON PATRICIA SONIA</t>
+          <t>C004174759 - BECERRA SOUZA JORGE ENRRIQUE</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>S17859698</t>
+          <t>S17848019</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -2001,7 +2001,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>77161</v>
+        <v>77156</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2035,12 +2035,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>C004203373</t>
+          <t>C004221411</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>C004203373 - LEVANO YARCURI ALBERTO RONALD</t>
+          <t>C004221411 - BELLO OBREGON PATRICIA SONIA</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>S17838640</t>
+          <t>S17859698</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -2100,7 +2100,7 @@
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2117,7 +2117,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>77541</v>
+        <v>77161</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2151,12 +2151,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>C004240376</t>
+          <t>C004203373</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>C004240376 - IGNACIO CARDENAS REGINALDA</t>
+          <t>C004203373 - LEVANO YARCURI ALBERTO RONALD</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>S17848813</t>
+          <t>S17838640</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Más confianza en la entrega</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr"/>
@@ -5481,16 +5481,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>97653</v>
+        <v>98051</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5515,12 +5515,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>C001104018</t>
+          <t>C001367095</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>C001104018 - ACERO SEGURA CECILIA NOEMI</t>
+          <t>C001367095 - JARA MATOS EXALTACION DE LA CRUZ</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>S17796713</t>
+          <t>S17794225</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -5554,11 +5554,11 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R44" t="n">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5585,28 +5585,28 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más capacitación</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>98051</v>
+        <v>97653</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5631,12 +5631,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>C001367095</t>
+          <t>C001104018</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>C001367095 - JARA MATOS EXALTACION DE LA CRUZ</t>
+          <t>C001104018 - ACERO SEGURA CECILIA NOEMI</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>S17794225</t>
+          <t>S17796713</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -5670,11 +5670,11 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R45" t="n">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="S45" t="inlineStr">
         <is>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5701,12 +5701,12 @@
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>Más capacitación</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr"/>
@@ -6177,16 +6177,16 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>66242</v>
+        <v>51627</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -6211,12 +6211,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>C004174114</t>
+          <t>C001747980</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>C004174114 - ENRIQUEZ FLORES MARLITH</t>
+          <t>C001747980 - CARRASCO JACINTO VILMA ADELA</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>S17740202</t>
+          <t>S17758670</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -6250,11 +6250,11 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R50" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="S50" t="inlineStr">
         <is>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -6276,12 +6276,12 @@
       <c r="X50" t="inlineStr"/>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Buscar productos</t>
         </is>
       </c>
       <c r="AA50" t="inlineStr">
@@ -6293,16 +6293,16 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>65527</v>
+        <v>58559</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6327,12 +6327,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>C001756035</t>
+          <t>C001727302</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>C001756035 - CAPCHA PROCEL FREDY</t>
+          <t>C001727302 - MERINO RUIZ ORESTES</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -6352,11 +6352,11 @@
         <v>46235</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>46247</v>
+        <v>46244</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>S17855887</t>
+          <t>S17743073</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -6366,11 +6366,11 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R51" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6392,12 +6392,12 @@
       <c r="X51" t="inlineStr"/>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Buscar productos</t>
         </is>
       </c>
       <c r="AA51" t="inlineStr">
@@ -6525,16 +6525,16 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>51627</v>
+        <v>65527</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>C001747980</t>
+          <t>C001756035</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>C001747980 - CARRASCO JACINTO VILMA ADELA</t>
+          <t>C001756035 - CAPCHA PROCEL FREDY</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -6584,11 +6584,11 @@
         <v>46235</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>S17758670</t>
+          <t>S17855887</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6598,11 +6598,11 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R53" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6624,12 +6624,12 @@
       <c r="X53" t="inlineStr"/>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>Buscar productos</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA53" t="inlineStr">
@@ -6641,16 +6641,16 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>58559</v>
+        <v>66242</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6675,12 +6675,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>C001727302</t>
+          <t>C004174114</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>C001727302 - MERINO RUIZ ORESTES</t>
+          <t>C004174114 - ENRIQUEZ FLORES MARLITH</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>S17743073</t>
+          <t>S17740202</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6714,11 +6714,11 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R54" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
@@ -6727,7 +6727,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6740,12 +6740,12 @@
       <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>Buscar productos</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
@@ -6873,16 +6873,16 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>37609</v>
+        <v>40761</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6907,12 +6907,12 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>C001678394</t>
+          <t>C001693228</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>C001678394 - CHAMPI OSCCO NATIVIDAD</t>
+          <t>C001693228 - ASENCIO MUÑOZ FABIAN VICTOR</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6932,11 +6932,11 @@
         <v>46235</v>
       </c>
       <c r="N56" s="3" t="n">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>S17770575</t>
+          <t>S17856541</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6946,11 +6946,11 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R56" t="n">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="S56" t="inlineStr">
         <is>
@@ -6959,7 +6959,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6972,17 +6972,17 @@
       <c r="X56" t="inlineStr"/>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
-          <t>Revisar despacho</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>Más productos disponibles</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr"/>
@@ -7221,16 +7221,16 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>40761</v>
+        <v>37609</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7255,12 +7255,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>C001693228</t>
+          <t>C001678394</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>C001693228 - ASENCIO MUÑOZ FABIAN VICTOR</t>
+          <t>C001678394 - CHAMPI OSCCO NATIVIDAD</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -7280,11 +7280,11 @@
         <v>46235</v>
       </c>
       <c r="N59" s="3" t="n">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>S17856541</t>
+          <t>S17770575</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -7294,11 +7294,11 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R59" t="n">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="S59" t="inlineStr">
         <is>
@@ -7307,7 +7307,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -7320,17 +7320,17 @@
       <c r="X59" t="inlineStr"/>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Revisar despacho</t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más productos disponibles</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr"/>
@@ -8369,7 +8369,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2938</v>
+        <v>2991</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -8403,12 +8403,12 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>C000656341</t>
+          <t>C001015412</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>C000656341 - ROSALES MANRIQUE MARIA</t>
+          <t>C001015412 - MAMANI COLCA EPIFANIA</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -8432,7 +8432,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>S17794159</t>
+          <t>S17782941</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -8455,7 +8455,7 @@
       </c>
       <c r="T69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
         </is>
       </c>
       <c r="U69" t="inlineStr">
@@ -8478,14 +8478,14 @@
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t>Más confianza en la entrega</t>
+          <t>Apoyo del vendedor</t>
         </is>
       </c>
       <c r="AB69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>2939</v>
+        <v>2938</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -8519,12 +8519,12 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>C000656485</t>
+          <t>C000656341</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>C000656485 - HUAMAN SULCARAYME LUCIANO</t>
+          <t>C000656341 - ROSALES MANRIQUE MARIA</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>S17776572</t>
+          <t>S17794159</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -8584,7 +8584,7 @@
       <c r="X70" t="inlineStr"/>
       <c r="Y70" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z70" t="inlineStr">
@@ -8601,7 +8601,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2991</v>
+        <v>2939</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -8635,12 +8635,12 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>C001015412</t>
+          <t>C000656485</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>C001015412 - MAMANI COLCA EPIFANIA</t>
+          <t>C000656485 - HUAMAN SULCARAYME LUCIANO</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>S17782941</t>
+          <t>S17776572</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="T71" t="inlineStr">
         <is>
-          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U71" t="inlineStr">
@@ -8700,7 +8700,7 @@
       <c r="X71" t="inlineStr"/>
       <c r="Y71" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z71" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>Apoyo del vendedor</t>
+          <t>Más confianza en la entrega</t>
         </is>
       </c>
       <c r="AB71" t="inlineStr"/>
@@ -9877,16 +9877,16 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>40599</v>
+        <v>37770</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9911,12 +9911,12 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>C001633200</t>
+          <t>C001643938</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>C001633200 - LEON GAMARRA MIRIAN CASILDA</t>
+          <t>C001643938 - MENDOZA ALVARADO MARIANELLA</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9936,11 +9936,11 @@
         <v>46235</v>
       </c>
       <c r="N82" s="3" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>S17764183</t>
+          <t>S17780003</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -9950,11 +9950,11 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R82" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="S82" t="inlineStr">
         <is>
@@ -9963,7 +9963,7 @@
       </c>
       <c r="T82" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
         </is>
       </c>
       <c r="U82" t="inlineStr">
@@ -9981,19 +9981,19 @@
       </c>
       <c r="Z82" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más capacitación</t>
         </is>
       </c>
       <c r="AB82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>40760</v>
+        <v>38632</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -10027,12 +10027,12 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>C001685996</t>
+          <t>C001662048</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>C001685996 - PALOMINO VALDERRAMA MARIA CRISTINA</t>
+          <t>C001662048 - LOPEZ LOPEZ JUDIHT SONIA</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -10052,11 +10052,11 @@
         <v>46235</v>
       </c>
       <c r="N83" s="3" t="n">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>S17749155</t>
+          <t>S17846214</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="T83" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Otros motivos</t>
         </is>
       </c>
       <c r="U83" t="inlineStr">
@@ -10092,7 +10092,7 @@
       <c r="X83" t="inlineStr"/>
       <c r="Y83" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z83" t="inlineStr">
@@ -10109,16 +10109,16 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>40616</v>
+        <v>40599</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -10143,12 +10143,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>C001710781</t>
+          <t>C001633200</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>C001710781 - IDROGO VEGA MARIA ERLA</t>
+          <t>C001633200 - LEON GAMARRA MIRIAN CASILDA</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -10168,11 +10168,11 @@
         <v>46235</v>
       </c>
       <c r="N84" s="3" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>S17788163</t>
+          <t>S17764183</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -10182,11 +10182,11 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R84" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="S84" t="inlineStr">
         <is>
@@ -10195,7 +10195,7 @@
       </c>
       <c r="T84" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U84" t="inlineStr">
@@ -10213,28 +10213,28 @@
       </c>
       <c r="Z84" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>Más capacitación</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>37770</v>
+        <v>40760</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -10259,12 +10259,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>C001643938</t>
+          <t>C001685996</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>C001643938 - MENDOZA ALVARADO MARIANELLA</t>
+          <t>C001685996 - PALOMINO VALDERRAMA MARIA CRISTINA</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -10284,11 +10284,11 @@
         <v>46235</v>
       </c>
       <c r="N85" s="3" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>S17780003</t>
+          <t>S17749155</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -10298,11 +10298,11 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R85" t="n">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="S85" t="inlineStr">
         <is>
@@ -10311,7 +10311,7 @@
       </c>
       <c r="T85" t="inlineStr">
         <is>
-          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U85" t="inlineStr">
@@ -10329,28 +10329,28 @@
       </c>
       <c r="Z85" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>Más capacitación</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>38632</v>
+        <v>40616</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -10375,12 +10375,12 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>C001662048</t>
+          <t>C001710781</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>C001662048 - LOPEZ LOPEZ JUDIHT SONIA</t>
+          <t>C001710781 - IDROGO VEGA MARIA ERLA</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -10400,11 +10400,11 @@
         <v>46235</v>
       </c>
       <c r="N86" s="3" t="n">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>S17846214</t>
+          <t>S17788163</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -10414,11 +10414,11 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R86" t="n">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="S86" t="inlineStr">
         <is>
@@ -10427,7 +10427,7 @@
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>Otros motivos</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U86" t="inlineStr">
@@ -10440,17 +10440,17 @@
       <c r="X86" t="inlineStr"/>
       <c r="Y86" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más capacitación</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr"/>
@@ -10573,16 +10573,16 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>46617</v>
+        <v>48512</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -10607,12 +10607,12 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>C001679008</t>
+          <t>C001675319</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>C001679008 - TINCO ZAMBRANO CARLOS EDWIN</t>
+          <t>C001675319 - ZAMORA CORDOVA YOSELIN</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10632,11 +10632,11 @@
         <v>46235</v>
       </c>
       <c r="N88" s="3" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>S17807288</t>
+          <t>S17752326</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -10646,11 +10646,11 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R88" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="S88" t="inlineStr">
         <is>
@@ -10677,7 +10677,7 @@
       </c>
       <c r="Z88" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA88" t="inlineStr">
@@ -10689,16 +10689,16 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>48512</v>
+        <v>46617</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10723,12 +10723,12 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>C001675319</t>
+          <t>C001679008</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>C001675319 - ZAMORA CORDOVA YOSELIN</t>
+          <t>C001679008 - TINCO ZAMBRANO CARLOS EDWIN</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10748,11 +10748,11 @@
         <v>46235</v>
       </c>
       <c r="N89" s="3" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>S17752326</t>
+          <t>S17807288</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -10762,11 +10762,11 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R89" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="S89" t="inlineStr">
         <is>
@@ -10793,7 +10793,7 @@
       </c>
       <c r="Z89" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA89" t="inlineStr">
@@ -10805,16 +10805,16 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>56043</v>
+        <v>65400</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -10839,12 +10839,12 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>C001649609</t>
+          <t>C001675344</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>C001649609 - IPARRAGUIRRE MORILLO DE QUEZADA NORIS</t>
+          <t>C001675344 - DULANTO HUAMAN SANDRA INES</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -10868,7 +10868,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>S17754247</t>
+          <t>S17750064</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -10878,11 +10878,11 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R90" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="S90" t="inlineStr">
         <is>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="T90" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U90" t="inlineStr">
@@ -10921,16 +10921,16 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>65400</v>
+        <v>56043</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -10955,12 +10955,12 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>C001675344</t>
+          <t>C001649609</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>C001675344 - DULANTO HUAMAN SANDRA INES</t>
+          <t>C001649609 - IPARRAGUIRRE MORILLO DE QUEZADA NORIS</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -10984,7 +10984,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>S17750064</t>
+          <t>S17754247</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -10994,11 +10994,11 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R91" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="S91" t="inlineStr">
         <is>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="T91" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U91" t="inlineStr">
@@ -11501,16 +11501,16 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>89885</v>
+        <v>89277</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -11535,12 +11535,12 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>C001748759</t>
+          <t>C001714772</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>C001748759 - AYALA MARIANO CARMEN MILAGROS</t>
+          <t>C001714772 - OROSCO RIOS RICHARD NICOLAS</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -11564,7 +11564,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>S17704475</t>
+          <t>S17693015</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
@@ -11574,11 +11574,11 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R96" t="n">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="S96" t="inlineStr">
         <is>
@@ -11587,7 +11587,7 @@
       </c>
       <c r="T96" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U96" t="inlineStr">
@@ -11600,33 +11600,33 @@
       <c r="X96" t="inlineStr"/>
       <c r="Y96" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
-          <t>Revisar despacho</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>Más productos disponibles</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>89277</v>
+        <v>89285</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -11651,12 +11651,12 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>C001714772</t>
+          <t>C001667402</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>C001714772 - OROSCO RIOS RICHARD NICOLAS</t>
+          <t>C001667402 - BAZAN APONTE GLORIA CRISTINA</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -11676,11 +11676,11 @@
         <v>46235</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46241</v>
+        <v>46245</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>S17693015</t>
+          <t>S17783871</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -11690,11 +11690,11 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R97" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="S97" t="inlineStr">
         <is>
@@ -11703,7 +11703,7 @@
       </c>
       <c r="T97" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U97" t="inlineStr">
@@ -11716,12 +11716,12 @@
       <c r="X97" t="inlineStr"/>
       <c r="Y97" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA97" t="inlineStr">
@@ -11733,16 +11733,16 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>89285</v>
+        <v>87710</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -11767,12 +11767,12 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>C001667402</t>
+          <t>C004180684</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>C001667402 - BAZAN APONTE GLORIA CRISTINA</t>
+          <t>C004180684 - HUAIRA BOZA EFRAIN</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -11792,11 +11792,11 @@
         <v>46235</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>S17783871</t>
+          <t>S17754546</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -11806,11 +11806,11 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R98" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="S98" t="inlineStr">
         <is>
@@ -11837,7 +11837,7 @@
       </c>
       <c r="Z98" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA98" t="inlineStr">
@@ -11965,16 +11965,16 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>87710</v>
+        <v>89885</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -11999,12 +11999,12 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>C004180684</t>
+          <t>C001748759</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>C004180684 - HUAIRA BOZA EFRAIN</t>
+          <t>C001748759 - AYALA MARIANO CARMEN MILAGROS</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -12024,11 +12024,11 @@
         <v>46235</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46244</v>
+        <v>46241</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>S17754546</t>
+          <t>S17704475</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -12038,11 +12038,11 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R100" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="S100" t="inlineStr">
         <is>
@@ -12069,12 +12069,12 @@
       </c>
       <c r="Z100" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Revisar despacho</t>
         </is>
       </c>
       <c r="AA100" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más productos disponibles</t>
         </is>
       </c>
       <c r="AB100" t="inlineStr"/>
@@ -12777,16 +12777,16 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>44559</v>
+        <v>42183</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12811,12 +12811,12 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>C001703595</t>
+          <t>C001685503</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>C001703595 - ORTIZ CACERES DE ZELADA DINA</t>
+          <t>C001685503 - ROQUE LOPEZ CARLOS AUGUSTO</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -12836,11 +12836,11 @@
         <v>46235</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>S17682074</t>
+          <t>S17738117</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
@@ -12850,11 +12850,11 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R107" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="S107" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
       </c>
       <c r="T107" t="inlineStr">
         <is>
-          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U107" t="inlineStr">
@@ -12881,28 +12881,28 @@
       </c>
       <c r="Z107" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>Más productos disponibles</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>35162</v>
+        <v>44559</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -12927,12 +12927,12 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>C001670996</t>
+          <t>C001703595</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>C001670996 - TIENDAS SOTHU S.A.C.</t>
+          <t>C001703595 - ORTIZ CACERES DE ZELADA DINA</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -12952,11 +12952,11 @@
         <v>46235</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46245</v>
+        <v>46241</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>S17783575</t>
+          <t>S17682074</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
@@ -12966,11 +12966,11 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R108" t="n">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="S108" t="inlineStr">
         <is>
@@ -12979,7 +12979,7 @@
       </c>
       <c r="T108" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
         </is>
       </c>
       <c r="U108" t="inlineStr">
@@ -12997,12 +12997,12 @@
       </c>
       <c r="Z108" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA108" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más productos disponibles</t>
         </is>
       </c>
       <c r="AB108" t="inlineStr"/>
@@ -13125,16 +13125,16 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>42183</v>
+        <v>35162</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -13159,12 +13159,12 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>C001685503</t>
+          <t>C001670996</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>C001685503 - ROQUE LOPEZ CARLOS AUGUSTO</t>
+          <t>C001670996 - TIENDAS SOTHU S.A.C.</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -13184,11 +13184,11 @@
         <v>46235</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>S17738117</t>
+          <t>S17783575</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -13198,11 +13198,11 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R110" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="S110" t="inlineStr">
         <is>
@@ -13229,7 +13229,7 @@
       </c>
       <c r="Z110" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA110" t="inlineStr">
@@ -14053,16 +14053,16 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>10702</v>
+        <v>13430</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -14087,12 +14087,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>C001014639</t>
+          <t>C001317592</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>C001014639 - QUISPE SIHUACOLLO MARTHA JIMENA</t>
+          <t>C001317592 - FLORES CERNA LIZ MARIELA</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -14112,11 +14112,11 @@
         <v>46235</v>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46245</v>
+        <v>46241</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>S17796539</t>
+          <t>S17678786</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -14126,11 +14126,11 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R118" t="n">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="S118" t="inlineStr">
         <is>
@@ -14139,7 +14139,7 @@
       </c>
       <c r="T118" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
         </is>
       </c>
       <c r="U118" t="inlineStr">
@@ -14157,19 +14157,19 @@
       </c>
       <c r="Z118" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Revisar despacho</t>
         </is>
       </c>
       <c r="AA118" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más capacitación</t>
         </is>
       </c>
       <c r="AB118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>15025</v>
+        <v>10702</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -14203,12 +14203,12 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>C001337157</t>
+          <t>C001014639</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>C001337157 - VASQUEZ QUISPE ANTHONY FRANK</t>
+          <t>C001014639 - QUISPE SIHUACOLLO MARTHA JIMENA</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -14232,7 +14232,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>S17779834</t>
+          <t>S17796539</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -14285,16 +14285,16 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>13430</v>
+        <v>15025</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -14319,12 +14319,12 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>C001317592</t>
+          <t>C001337157</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>C001317592 - FLORES CERNA LIZ MARIELA</t>
+          <t>C001337157 - VASQUEZ QUISPE ANTHONY FRANK</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -14344,11 +14344,11 @@
         <v>46235</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46241</v>
+        <v>46245</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>S17678786</t>
+          <t>S17779834</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -14358,11 +14358,11 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R120" t="n">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -14371,7 +14371,7 @@
       </c>
       <c r="T120" t="inlineStr">
         <is>
-          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U120" t="inlineStr">
@@ -14389,12 +14389,12 @@
       </c>
       <c r="Z120" t="inlineStr">
         <is>
-          <t>Revisar despacho</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA120" t="inlineStr">
         <is>
-          <t>Más capacitación</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB120" t="inlineStr"/>
@@ -14865,16 +14865,16 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>4293</v>
+        <v>3197</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -14899,12 +14899,12 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>C000663717</t>
+          <t>C000663105</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>C000663717 - PALOMINO PALOMINO ZOSIMO</t>
+          <t>C000663105 - FLORES VILLANUEVA SISTO</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -14924,11 +14924,11 @@
         <v>46235</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>S17625225</t>
+          <t>S17685537</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -14938,11 +14938,11 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R125" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="S125" t="inlineStr">
         <is>
@@ -14951,7 +14951,7 @@
       </c>
       <c r="T125" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U125" t="inlineStr">
@@ -14969,7 +14969,7 @@
       </c>
       <c r="Z125" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA125" t="inlineStr">
@@ -15097,16 +15097,16 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>3197</v>
+        <v>6656</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -15131,12 +15131,12 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>C000663105</t>
+          <t>C000659327</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>C000663105 - FLORES VILLANUEVA SISTO</t>
+          <t>C000659327 - ATAPOMA BEIZAGA BRENDA DEL ROCIO</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -15156,11 +15156,11 @@
         <v>46235</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>S17685537</t>
+          <t>S17666472</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
@@ -15170,11 +15170,11 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R127" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="S127" t="inlineStr">
         <is>
@@ -15201,7 +15201,7 @@
       </c>
       <c r="Z127" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA127" t="inlineStr">
@@ -15213,7 +15213,7 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>6656</v>
+        <v>4293</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -15247,12 +15247,12 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>C000659327</t>
+          <t>C000663717</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>C000659327 - ATAPOMA BEIZAGA BRENDA DEL ROCIO</t>
+          <t>C000663717 - PALOMINO PALOMINO ZOSIMO</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -15272,11 +15272,11 @@
         <v>46235</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>S17666472</t>
+          <t>S17625225</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="T128" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U128" t="inlineStr">
@@ -15677,16 +15677,16 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>38049</v>
+        <v>34091</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -15711,12 +15711,12 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>C001572085</t>
+          <t>C001552031</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>C001572085 - MAMANI MAMANI ROSA ELA</t>
+          <t>C001552031 - VENTURA FLORES PERCY RODRIGO</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -15736,11 +15736,11 @@
         <v>46235</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46244</v>
+        <v>46241</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>S17752025</t>
+          <t>S17702876</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -15750,11 +15750,11 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R132" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
@@ -15763,7 +15763,7 @@
       </c>
       <c r="T132" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U132" t="inlineStr">
@@ -15776,12 +15776,12 @@
       <c r="X132" t="inlineStr"/>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z132" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA132" t="inlineStr">
@@ -15793,16 +15793,16 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>34091</v>
+        <v>38049</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -15827,12 +15827,12 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>C001552031</t>
+          <t>C001572085</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>C001552031 - VENTURA FLORES PERCY RODRIGO</t>
+          <t>C001572085 - MAMANI MAMANI ROSA ELA</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -15852,11 +15852,11 @@
         <v>46235</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>S17702876</t>
+          <t>S17752025</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
@@ -15866,11 +15866,11 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R133" t="n">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="S133" t="inlineStr">
         <is>
@@ -15879,7 +15879,7 @@
       </c>
       <c r="T133" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U133" t="inlineStr">
@@ -15892,12 +15892,12 @@
       <c r="X133" t="inlineStr"/>
       <c r="Y133" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z133" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA133" t="inlineStr">
@@ -16025,7 +16025,7 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>59251</v>
+        <v>63206</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -16059,12 +16059,12 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>C004033907</t>
+          <t>C001746377</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>C004033907 - LLAMPI PFUÑO JULIANA</t>
+          <t>C001746377 - CHUJANDAMA GARCIA DE ROSALES CARMEN ROSA</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -16084,11 +16084,11 @@
         <v>46235</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>S17623020</t>
+          <t>S17704214</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
@@ -16111,7 +16111,7 @@
       </c>
       <c r="T135" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U135" t="inlineStr">
@@ -16141,7 +16141,7 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>63206</v>
+        <v>59251</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -16175,12 +16175,12 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>C001746377</t>
+          <t>C004033907</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>C001746377 - CHUJANDAMA GARCIA DE ROSALES CARMEN ROSA</t>
+          <t>C004033907 - LLAMPI PFUÑO JULIANA</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -16200,11 +16200,11 @@
         <v>46235</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>S17704214</t>
+          <t>S17623020</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
@@ -16227,7 +16227,7 @@
       </c>
       <c r="T136" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U136" t="inlineStr">
@@ -19273,16 +19273,16 @@
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>35198</v>
+        <v>33337</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -19307,12 +19307,12 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>C001647244</t>
+          <t>C001628789</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>C001647244 - HUERTA LEON JORGE EDUARDO</t>
+          <t>C001628789 - VEGA VEGA YELITZA ANGELICA</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -19336,7 +19336,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>S17584287</t>
+          <t>S17609283</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -19346,11 +19346,11 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R163" t="n">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="S163" t="inlineStr">
         <is>
@@ -19377,28 +19377,28 @@
       </c>
       <c r="Z163" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA163" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más productos disponibles</t>
         </is>
       </c>
       <c r="AB163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>34876</v>
+        <v>35198</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -19423,12 +19423,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>C001557347</t>
+          <t>C001647244</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>C001557347 - MAGUINA MALLQUI NANCY VICTORIA</t>
+          <t>C001647244 - HUERTA LEON JORGE EDUARDO</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -19448,11 +19448,11 @@
         <v>46235</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46242</v>
+        <v>46238</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>S17721156</t>
+          <t>S17584287</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -19462,11 +19462,11 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R164" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="S164" t="inlineStr">
         <is>
@@ -19475,7 +19475,7 @@
       </c>
       <c r="T164" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U164" t="inlineStr">
@@ -19493,7 +19493,7 @@
       </c>
       <c r="Z164" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA164" t="inlineStr">
@@ -19505,7 +19505,7 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>25535</v>
+        <v>34876</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -19539,12 +19539,12 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>C001535577</t>
+          <t>C001557347</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>C001535577 - TURPO HUILLCA FORTUNATA</t>
+          <t>C001557347 - MAGUINA MALLQUI NANCY VICTORIA</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -19564,11 +19564,11 @@
         <v>46235</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46238</v>
+        <v>46242</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>S17609102</t>
+          <t>S17721156</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
@@ -19604,7 +19604,7 @@
       <c r="X165" t="inlineStr"/>
       <c r="Y165" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z165" t="inlineStr">
@@ -19621,16 +19621,16 @@
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>28718</v>
+        <v>25535</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -19655,12 +19655,12 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>C001506593</t>
+          <t>C001535577</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>C001506593 - DIAZ GARRIDO BLANCA MARIA</t>
+          <t>C001535577 - TURPO HUILLCA FORTUNATA</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -19680,11 +19680,11 @@
         <v>46235</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>S17662166</t>
+          <t>S17609102</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
@@ -19694,11 +19694,11 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R166" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="S166" t="inlineStr">
         <is>
@@ -19707,7 +19707,7 @@
       </c>
       <c r="T166" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U166" t="inlineStr">
@@ -19720,7 +19720,7 @@
       <c r="X166" t="inlineStr"/>
       <c r="Y166" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z166" t="inlineStr">
@@ -19737,16 +19737,16 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>33337</v>
+        <v>28718</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -19771,12 +19771,12 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>C001628789</t>
+          <t>C001506593</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>C001628789 - VEGA VEGA YELITZA ANGELICA</t>
+          <t>C001506593 - DIAZ GARRIDO BLANCA MARIA</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -19796,11 +19796,11 @@
         <v>46235</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46238</v>
+        <v>46240</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>S17609283</t>
+          <t>S17662166</t>
         </is>
       </c>
       <c r="P167" t="inlineStr">
@@ -19810,11 +19810,11 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R167" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="S167" t="inlineStr">
         <is>
@@ -19841,12 +19841,12 @@
       </c>
       <c r="Z167" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA167" t="inlineStr">
         <is>
-          <t>Más productos disponibles</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB167" t="inlineStr"/>
@@ -21221,16 +21221,16 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>29124</v>
+        <v>26034</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -21255,12 +21255,12 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>C001525470</t>
+          <t>C001527992</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>C001525470 - IMAN CCAIHUARI MIRELLA INES</t>
+          <t>C001527992 - NEYRA RODRIGUEZ CENIA</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -21280,11 +21280,11 @@
         <v>46235</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>S17581044</t>
+          <t>S17550155</t>
         </is>
       </c>
       <c r="P180" t="inlineStr">
@@ -21294,11 +21294,11 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R180" t="n">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="S180" t="inlineStr">
         <is>
@@ -21307,7 +21307,7 @@
       </c>
       <c r="T180" t="inlineStr">
         <is>
-          <t>No cuenta con presupuesto disponible en ese momento.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U180" t="inlineStr">
@@ -21320,33 +21320,33 @@
       <c r="X180" t="inlineStr"/>
       <c r="Y180" t="inlineStr">
         <is>
-          <t>Muy dispuesto</t>
+          <t>Algo dispuesto</t>
         </is>
       </c>
       <c r="Z180" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA180" t="inlineStr">
         <is>
-          <t>Más productos disponibles</t>
+          <t>Más confianza en la entrega</t>
         </is>
       </c>
       <c r="AB180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>26034</v>
+        <v>27335</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -21371,12 +21371,12 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>C001527992</t>
+          <t>C001519043</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>C001527992 - NEYRA RODRIGUEZ CENIA</t>
+          <t>C001519043 - CALLEGARI MUNIVE HUGO JEAMPIERE</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -21396,11 +21396,11 @@
         <v>46235</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46237</v>
+        <v>46247</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>S17550155</t>
+          <t>S17838829</t>
         </is>
       </c>
       <c r="P181" t="inlineStr">
@@ -21410,11 +21410,11 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R181" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="S181" t="inlineStr">
         <is>
@@ -21423,7 +21423,7 @@
       </c>
       <c r="T181" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U181" t="inlineStr">
@@ -21436,33 +21436,33 @@
       <c r="X181" t="inlineStr"/>
       <c r="Y181" t="inlineStr">
         <is>
-          <t>Algo dispuesto</t>
+          <t>Muy dispuesto</t>
         </is>
       </c>
       <c r="Z181" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA181" t="inlineStr">
         <is>
-          <t>Más confianza en la entrega</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>27335</v>
+        <v>29124</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -21487,12 +21487,12 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>C001519043</t>
+          <t>C001525470</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>C001519043 - CALLEGARI MUNIVE HUGO JEAMPIERE</t>
+          <t>C001525470 - IMAN CCAIHUARI MIRELLA INES</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -21512,11 +21512,11 @@
         <v>46235</v>
       </c>
       <c r="N182" s="3" t="n">
-        <v>46247</v>
+        <v>46238</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>S17838829</t>
+          <t>S17581044</t>
         </is>
       </c>
       <c r="P182" t="inlineStr">
@@ -21526,11 +21526,11 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R182" t="n">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="S182" t="inlineStr">
         <is>
@@ -21539,7 +21539,7 @@
       </c>
       <c r="T182" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>No cuenta con presupuesto disponible en ese momento.</t>
         </is>
       </c>
       <c r="U182" t="inlineStr">
@@ -21557,12 +21557,12 @@
       </c>
       <c r="Z182" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA182" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más productos disponibles</t>
         </is>
       </c>
       <c r="AB182" t="inlineStr"/>
@@ -22265,7 +22265,7 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>54249</v>
+        <v>62539</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -22299,12 +22299,12 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>C001739985</t>
+          <t>C001765058</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>C001739985 - MARCOS CELEDONIO ELISABETH ORFA</t>
+          <t>C001765058 - VERAMENDI RAMIREZ OLGA DINA</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -22324,11 +22324,11 @@
         <v>46235</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>S17669600</t>
+          <t>S17759804</t>
         </is>
       </c>
       <c r="P189" t="inlineStr">
@@ -22381,7 +22381,7 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>53844</v>
+        <v>59953</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -22415,12 +22415,12 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>C001727562</t>
+          <t>C001756391</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>C001727562 - ROSALES CASTILLO REYNA MARCELINA</t>
+          <t>C001756391 - MARQUEZ MARTEL CARMEN LUISA</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -22440,11 +22440,11 @@
         <v>46235</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>S17678384</t>
+          <t>S17576336</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
@@ -22497,7 +22497,7 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>57185</v>
+        <v>58928</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -22531,12 +22531,12 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>C001737715</t>
+          <t>C001755995</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>C001737715 - RICSE RODRIGUEZ ROSMERY TARCILA</t>
+          <t>C001755995 - ORTEGA MONTESINOS IRMA DORIS</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -22556,11 +22556,11 @@
         <v>46235</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46239</v>
+        <v>46237</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>S17640201</t>
+          <t>S17561870</t>
         </is>
       </c>
       <c r="P191" t="inlineStr">
@@ -22583,7 +22583,7 @@
       </c>
       <c r="T191" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="U191" t="inlineStr">
@@ -22613,16 +22613,16 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>58928</v>
+        <v>54249</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>76023169</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -22647,12 +22647,12 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>C001755995</t>
+          <t>C001739985</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>C001755995 - ORTEGA MONTESINOS IRMA DORIS</t>
+          <t>C001739985 - MARCOS CELEDONIO ELISABETH ORFA</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -22672,11 +22672,11 @@
         <v>46235</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46237</v>
+        <v>46240</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>S17561870</t>
+          <t>S17669600</t>
         </is>
       </c>
       <c r="P192" t="inlineStr">
@@ -22686,11 +22686,11 @@
       </c>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R192" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="S192" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
       </c>
       <c r="T192" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U192" t="inlineStr">
@@ -22717,7 +22717,7 @@
       </c>
       <c r="Z192" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA192" t="inlineStr">
@@ -22729,16 +22729,16 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>62539</v>
+        <v>53844</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>ESTEFANY LUCY RAMOS AYMITUMA</t>
+          <t>BRYAN SMITH PAREDES MALCA</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>76023169</t>
+          <t>75315055</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -22763,12 +22763,12 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>C001765058</t>
+          <t>C001727562</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>C001765058 - VERAMENDI RAMIREZ OLGA DINA</t>
+          <t>C001727562 - ROSALES CASTILLO REYNA MARCELINA</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -22788,11 +22788,11 @@
         <v>46235</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46244</v>
+        <v>46241</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>S17759804</t>
+          <t>S17678384</t>
         </is>
       </c>
       <c r="P193" t="inlineStr">
@@ -22802,11 +22802,11 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>76023169LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R193" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="S193" t="inlineStr">
         <is>
@@ -22815,7 +22815,7 @@
       </c>
       <c r="T193" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
         </is>
       </c>
       <c r="U193" t="inlineStr">
@@ -22833,28 +22833,28 @@
       </c>
       <c r="Z193" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Agregar productos al carrito</t>
         </is>
       </c>
       <c r="AA193" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más productos disponibles</t>
         </is>
       </c>
       <c r="AB193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>59953</v>
+        <v>57185</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>BRYAN SMITH PAREDES MALCA</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>75315055</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -22879,12 +22879,12 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>C001756391</t>
+          <t>C001737715</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>C001756391 - MARQUEZ MARTEL CARMEN LUISA</t>
+          <t>C001737715 - RICSE RODRIGUEZ ROSMERY TARCILA</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -22904,11 +22904,11 @@
         <v>46235</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>S17576336</t>
+          <t>S17640201</t>
         </is>
       </c>
       <c r="P194" t="inlineStr">
@@ -22918,11 +22918,11 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>75315055LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R194" t="n">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="S194" t="inlineStr">
         <is>
@@ -22931,7 +22931,7 @@
       </c>
       <c r="T194" t="inlineStr">
         <is>
-          <t>Está esperando promociones, descuentos o condiciones más favorables.</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U194" t="inlineStr">
@@ -22949,12 +22949,12 @@
       </c>
       <c r="Z194" t="inlineStr">
         <is>
-          <t>Agregar productos al carrito</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA194" t="inlineStr">
         <is>
-          <t>Más productos disponibles</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB194" t="inlineStr"/>
@@ -25165,7 +25165,7 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>73062</v>
+        <v>73840</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -25199,12 +25199,12 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>C004093718</t>
+          <t>C004048445</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>C004093718 - LOPEZ SANCHEZ JOSE ANTONIO</t>
+          <t>C004048445 - SARAZU GAMARRA CARLOS MAGNO</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -25224,11 +25224,11 @@
         <v>46235</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46241</v>
+        <v>46238</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>S17680195</t>
+          <t>S17598739</t>
         </is>
       </c>
       <c r="P214" t="inlineStr">
@@ -25281,7 +25281,7 @@
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>73840</v>
+        <v>73062</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -25315,12 +25315,12 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>C004048445</t>
+          <t>C004093718</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>C004048445 - SARAZU GAMARRA CARLOS MAGNO</t>
+          <t>C004093718 - LOPEZ SANCHEZ JOSE ANTONIO</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -25340,11 +25340,11 @@
         <v>46235</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>S17598739</t>
+          <t>S17680195</t>
         </is>
       </c>
       <c r="P215" t="inlineStr">
@@ -25513,16 +25513,16 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>40179</v>
+        <v>38391</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>MARVIN MARCEL ACUÑA TORRES</t>
+          <t>SANDRA NIT HUAMAN CHILINGANO</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>43126649</t>
+          <t>9984323</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -25547,12 +25547,12 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>C001649854</t>
+          <t>C001627779</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>C001649854 - ESPINOZA DIAZ ROBERTO EDGAR</t>
+          <t>C001627779 - SARAZU GAMARRA ELIDA MARGARITA</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -25572,11 +25572,11 @@
         <v>46235</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>S17686520</t>
+          <t>S17573965</t>
         </is>
       </c>
       <c r="P217" t="inlineStr">
@@ -25586,11 +25586,11 @@
       </c>
       <c r="Q217" t="inlineStr">
         <is>
-          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R217" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="S217" t="inlineStr">
         <is>
@@ -25599,7 +25599,7 @@
       </c>
       <c r="T217" t="inlineStr">
         <is>
-          <t>Prefiere negociar con el vendedor</t>
+          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
         </is>
       </c>
       <c r="U217" t="inlineStr">
@@ -25617,28 +25617,28 @@
       </c>
       <c r="Z217" t="inlineStr">
         <is>
-          <t>Ninguna, entendió correctamente</t>
+          <t>Ver promociones</t>
         </is>
       </c>
       <c r="AA217" t="inlineStr">
         <is>
-          <t>Más confianza en la entrega</t>
+          <t>Mejores promociones</t>
         </is>
       </c>
       <c r="AB217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>38391</v>
+        <v>40179</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>SANDRA NIT HUAMAN CHILINGANO</t>
+          <t>MARVIN MARCEL ACUÑA TORRES</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>9984323</t>
+          <t>43126649</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -25663,12 +25663,12 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>C001627779</t>
+          <t>C001649854</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>C001627779 - SARAZU GAMARRA ELIDA MARGARITA</t>
+          <t>C001649854 - ESPINOZA DIAZ ROBERTO EDGAR</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -25688,11 +25688,11 @@
         <v>46235</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46237</v>
+        <v>46241</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>S17573965</t>
+          <t>S17686520</t>
         </is>
       </c>
       <c r="P218" t="inlineStr">
@@ -25702,11 +25702,11 @@
       </c>
       <c r="Q218" t="inlineStr">
         <is>
-          <t>9984323LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
+          <t>43126649LIMAVIZARRETA SANCHEZ, ELIZABETH DAYANA1000001534</t>
         </is>
       </c>
       <c r="R218" t="n">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="S218" t="inlineStr">
         <is>
@@ -25715,7 +25715,7 @@
       </c>
       <c r="T218" t="inlineStr">
         <is>
-          <t>Tiene stock suficiente y quiere evitar sobre inventario.</t>
+          <t>Prefiere negociar con el vendedor</t>
         </is>
       </c>
       <c r="U218" t="inlineStr">
@@ -25733,12 +25733,12 @@
       </c>
       <c r="Z218" t="inlineStr">
         <is>
-          <t>Ver promociones</t>
+          <t>Ninguna, entendió correctamente</t>
         </is>
       </c>
       <c r="AA218" t="inlineStr">
         <is>
-          <t>Mejores promociones</t>
+          <t>Más confianza en la entrega</t>
         </is>
       </c>
       <c r="AB218" t="inlineStr"/>

</xml_diff>